<commit_message>
Done LSU module and testbench
 Load/Store Unit (LSU) Completed and Tested

Approximately 147 million randomized and critical end-point tests were successful. The module was deemed stable, and the LSU was fully completed.
</commit_message>
<xml_diff>
--- a/Documents/LSU Sub-Opcode Table.xlsx
+++ b/Documents/LSU Sub-Opcode Table.xlsx
@@ -24,13 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="51">
-  <si>
-    <t>OPCODE</t>
-  </si>
-  <si>
-    <t>SUB-OPCODE</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="61">
   <si>
     <t>Operation</t>
   </si>
@@ -134,12 +128,6 @@
     <t>Move</t>
   </si>
   <si>
-    <t>SLRP</t>
-  </si>
-  <si>
-    <t>Select Register Page</t>
-  </si>
-  <si>
     <t>LDI</t>
   </si>
   <si>
@@ -152,18 +140,12 @@
     <t>Store Immediately</t>
   </si>
   <si>
-    <t>EDB</t>
-  </si>
-  <si>
     <t>Source</t>
   </si>
   <si>
     <t>Target</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Register</t>
   </si>
   <si>
@@ -173,10 +155,58 @@
     <t>GPIO Reg</t>
   </si>
   <si>
-    <t>Controller</t>
-  </si>
-  <si>
     <t>Immediate</t>
+  </si>
+  <si>
+    <t>SMIO</t>
+  </si>
+  <si>
+    <t>Set Mode Input/Output</t>
+  </si>
+  <si>
+    <t>Null</t>
+  </si>
+  <si>
+    <t>OPCODE(ALU)</t>
+  </si>
+  <si>
+    <t>SUB-OPCODE(LSU)</t>
+  </si>
+  <si>
+    <t>JZ</t>
+  </si>
+  <si>
+    <t>Jump If Zero</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>JMP</t>
+  </si>
+  <si>
+    <t>Jump to an address</t>
+  </si>
+  <si>
+    <t>JNZ</t>
+  </si>
+  <si>
+    <t>Jump If Not Zero</t>
+  </si>
+  <si>
+    <t>CALL</t>
+  </si>
+  <si>
+    <t>Return From a Function</t>
+  </si>
+  <si>
+    <t>Call a Function</t>
+  </si>
+  <si>
+    <t>FuncReg</t>
+  </si>
+  <si>
+    <t>RET</t>
   </si>
 </sst>
 </file>
@@ -230,6 +260,21 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tablo1" displayName="Tablo1" ref="A1:F17" totalsRowShown="0">
+  <autoFilter ref="A1:F17"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="OPCODE(ALU)"/>
+    <tableColumn id="2" name="SUB-OPCODE(LSU)"/>
+    <tableColumn id="3" name="Operation Codename"/>
+    <tableColumn id="4" name="Operation"/>
+    <tableColumn id="5" name="Source"/>
+    <tableColumn id="6" name="Target"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium28" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -498,296 +543,358 @@
   <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.7109375" customWidth="1"/>
-    <col min="3" max="4" width="19.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" customWidth="1"/>
     <col min="5" max="6" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
       <c r="E1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="F3" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E4" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="F4" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F6" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F7" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E9" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F10" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E11" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="F11" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" t="s">
+        <v>43</v>
+      </c>
+      <c r="F12" t="s">
         <v>41</v>
-      </c>
-      <c r="E12" t="s">
-        <v>50</v>
-      </c>
-      <c r="F12" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>49</v>
+      </c>
+      <c r="D13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>14</v>
+      </c>
+      <c r="C14" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>15</v>
+      </c>
+      <c r="C15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="C16" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" t="s">
+        <v>58</v>
+      </c>
+      <c r="E16" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" t="s">
+        <v>57</v>
+      </c>
+      <c r="E17" t="s">
+        <v>59</v>
+      </c>
+      <c r="F17" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>